<commit_message>
Added consistent decimal places
</commit_message>
<xml_diff>
--- a/ecc_data_raw.xlsx
+++ b/ecc_data_raw.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10315"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10412"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/matthewv/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/matthewv/Desktop/ECC3479-/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{57CC65BB-E3D6-7E44-8C62-C4D509353F5C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9EB88BC1-B45C-6045-B801-DAF824CB0A89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="480" yWindow="1200" windowWidth="26400" windowHeight="15840" xr2:uid="{8A29026E-1C4A-8D46-A99E-EB38AD75A7CB}"/>
+    <workbookView xWindow="480" yWindow="800" windowWidth="26400" windowHeight="15840" xr2:uid="{8A29026E-1C4A-8D46-A99E-EB38AD75A7CB}"/>
   </bookViews>
   <sheets>
     <sheet name="Cleaned data" sheetId="1" r:id="rId1"/>
@@ -71,7 +71,7 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
     <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="164" formatCode="#,##0.0"/>
+    <numFmt numFmtId="166" formatCode="0.000"/>
   </numFmts>
   <fonts count="8" x14ac:knownFonts="1">
     <font>
@@ -158,24 +158,25 @@
       <alignment horizontal="right"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="3" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Currency" xfId="1" builtinId="4"/>
@@ -512,7 +513,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AF6A4F6A-0886-E340-AFA3-53C737302FD8}">
-  <dimension ref="A2:M25"/>
+  <dimension ref="A2:M22"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="3" width="12.5" bestFit="1" customWidth="1"/>
@@ -557,10 +558,12 @@
       <c r="A3">
         <v>2023</v>
       </c>
-      <c r="B3">
+      <c r="B3" s="6">
         <v>11.1</v>
       </c>
-      <c r="E3" s="3">
+      <c r="C3" s="6"/>
+      <c r="D3" s="6"/>
+      <c r="E3" s="5">
         <v>1.16435</v>
       </c>
       <c r="F3">
@@ -571,50 +574,50 @@
       <c r="A4">
         <v>2022</v>
       </c>
-      <c r="B4" s="1">
+      <c r="B4" s="11">
         <v>13.1</v>
       </c>
-      <c r="C4" s="1">
+      <c r="C4" s="11">
         <v>15.2</v>
       </c>
-      <c r="D4" s="1">
+      <c r="D4" s="11">
         <v>10</v>
       </c>
-      <c r="E4" s="6">
+      <c r="E4" s="7">
         <v>1.1268800000000001</v>
       </c>
-      <c r="F4" s="5">
+      <c r="F4" s="3">
         <v>2639.4</v>
       </c>
-      <c r="J4" s="4"/>
-      <c r="K4" s="4"/>
+      <c r="J4" s="2"/>
+      <c r="K4" s="2"/>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>2021</v>
       </c>
-      <c r="B5">
+      <c r="B5" s="6">
         <v>13.4</v>
       </c>
-      <c r="C5">
+      <c r="C5" s="6">
         <v>15.6</v>
       </c>
-      <c r="D5">
+      <c r="D5" s="6">
         <v>11.2</v>
       </c>
-      <c r="E5" s="6">
+      <c r="E5" s="7">
         <v>1.1035999999999999</v>
       </c>
       <c r="F5">
         <v>2098.1</v>
       </c>
-      <c r="G5" s="2">
+      <c r="G5" s="4">
         <v>53.7</v>
       </c>
-      <c r="H5" s="2">
+      <c r="H5" s="4">
         <v>62.3</v>
       </c>
-      <c r="I5" s="3">
+      <c r="I5" s="5">
         <v>46.6</v>
       </c>
     </row>
@@ -622,28 +625,28 @@
       <c r="A6">
         <v>2020</v>
       </c>
-      <c r="B6">
+      <c r="B6" s="6">
         <v>13.7</v>
       </c>
-      <c r="C6">
+      <c r="C6" s="6">
         <v>15.9</v>
       </c>
-      <c r="D6">
+      <c r="D6" s="6">
         <v>11.5</v>
       </c>
-      <c r="E6" s="6">
+      <c r="E6" s="7">
         <v>0.94964000000000004</v>
       </c>
       <c r="F6">
         <v>1560.6</v>
       </c>
-      <c r="G6" s="2">
+      <c r="G6" s="4">
         <v>55.9</v>
       </c>
-      <c r="H6" s="2">
+      <c r="H6" s="4">
         <v>64.400000000000006</v>
       </c>
-      <c r="I6" s="3">
+      <c r="I6" s="5">
         <v>48.9</v>
       </c>
     </row>
@@ -651,13 +654,13 @@
       <c r="A7">
         <v>2019</v>
       </c>
-      <c r="B7">
+      <c r="B7" s="6">
         <v>12.9</v>
       </c>
-      <c r="C7">
+      <c r="C7" s="6">
         <v>14.4</v>
       </c>
-      <c r="D7">
+      <c r="D7" s="6">
         <v>11.6</v>
       </c>
       <c r="E7" s="8">
@@ -666,13 +669,13 @@
       <c r="F7">
         <v>605.79999999999995</v>
       </c>
-      <c r="G7">
+      <c r="G7" s="6">
         <v>57.4</v>
       </c>
-      <c r="H7">
+      <c r="H7" s="6">
         <v>68.3</v>
       </c>
-      <c r="I7">
+      <c r="I7" s="6">
         <v>48.6</v>
       </c>
     </row>
@@ -680,13 +683,13 @@
       <c r="A8">
         <v>2016</v>
       </c>
-      <c r="B8">
+      <c r="B8" s="6">
         <v>14.2</v>
       </c>
-      <c r="C8">
+      <c r="C8" s="6">
         <v>16.3</v>
       </c>
-      <c r="D8">
+      <c r="D8" s="6">
         <v>12.3</v>
       </c>
       <c r="E8" s="8">
@@ -695,13 +698,13 @@
       <c r="F8">
         <v>388.8</v>
       </c>
-      <c r="G8">
+      <c r="G8" s="6">
         <v>58.5</v>
       </c>
-      <c r="H8">
+      <c r="H8" s="6">
         <v>71.7</v>
       </c>
-      <c r="I8">
+      <c r="I8" s="6">
         <v>47.8</v>
       </c>
     </row>
@@ -709,28 +712,28 @@
       <c r="A9">
         <v>2015</v>
       </c>
-      <c r="B9">
+      <c r="B9" s="6">
         <v>15.9</v>
       </c>
-      <c r="C9">
+      <c r="C9" s="6">
         <v>18.100000000000001</v>
       </c>
-      <c r="D9">
+      <c r="D9" s="6">
         <v>13.7</v>
       </c>
-      <c r="E9" s="6">
+      <c r="E9" s="7">
         <v>0.47008</v>
       </c>
       <c r="F9">
         <v>184</v>
       </c>
-      <c r="G9" s="2">
+      <c r="G9" s="4">
         <v>56.6</v>
       </c>
-      <c r="H9" s="2">
+      <c r="H9" s="4">
         <v>70.099999999999994</v>
       </c>
-      <c r="I9" s="3">
+      <c r="I9" s="5">
         <v>45.6</v>
       </c>
     </row>
@@ -738,13 +741,13 @@
       <c r="A10">
         <v>2013</v>
       </c>
-      <c r="B10">
+      <c r="B10" s="6">
         <v>16.399999999999999</v>
       </c>
-      <c r="C10">
+      <c r="C10" s="6">
         <v>16.8</v>
       </c>
-      <c r="D10">
+      <c r="D10" s="6">
         <v>12.7</v>
       </c>
       <c r="E10" s="8">
@@ -753,13 +756,13 @@
       <c r="F10">
         <v>369.5</v>
       </c>
-      <c r="G10">
+      <c r="G10" s="6">
         <v>57</v>
       </c>
-      <c r="H10">
+      <c r="H10" s="6">
         <v>73.2</v>
       </c>
-      <c r="I10">
+      <c r="I10" s="6">
         <v>43.9</v>
       </c>
     </row>
@@ -767,28 +770,28 @@
       <c r="A11">
         <v>2010</v>
       </c>
-      <c r="B11">
+      <c r="B11" s="6">
         <v>17.5</v>
       </c>
-      <c r="C11">
+      <c r="C11" s="6">
         <v>20.6</v>
       </c>
-      <c r="D11">
+      <c r="D11" s="6">
         <v>16.2</v>
       </c>
-      <c r="E11" s="7">
+      <c r="E11" s="9">
         <v>0.33267000000000002</v>
       </c>
       <c r="F11">
         <v>404.5</v>
       </c>
-      <c r="G11" s="2">
+      <c r="G11" s="4">
         <v>57.5</v>
       </c>
-      <c r="H11" s="2">
+      <c r="H11" s="4">
         <v>75.900000000000006</v>
       </c>
-      <c r="I11" s="3">
+      <c r="I11" s="5">
         <v>42.9</v>
       </c>
     </row>
@@ -796,19 +799,22 @@
       <c r="A12">
         <v>2009</v>
       </c>
-      <c r="E12" s="7">
+      <c r="B12" s="6"/>
+      <c r="C12" s="6"/>
+      <c r="D12" s="6"/>
+      <c r="E12" s="9">
         <v>0.25833</v>
       </c>
       <c r="F12">
         <v>457.1</v>
       </c>
-      <c r="G12" s="2">
+      <c r="G12" s="4">
         <v>58.2</v>
       </c>
-      <c r="H12" s="2">
+      <c r="H12" s="4">
         <v>75.7</v>
       </c>
-      <c r="I12" s="3">
+      <c r="I12" s="5">
         <v>44.4</v>
       </c>
     </row>
@@ -816,19 +822,22 @@
       <c r="A13">
         <v>2008</v>
       </c>
-      <c r="E13" s="7">
+      <c r="B13" s="6"/>
+      <c r="C13" s="6"/>
+      <c r="D13" s="6"/>
+      <c r="E13" s="9">
         <v>0.2545</v>
       </c>
       <c r="F13">
         <v>269.39999999999998</v>
       </c>
-      <c r="G13" s="2">
+      <c r="G13" s="4">
         <v>58.6</v>
       </c>
-      <c r="H13" s="2">
+      <c r="H13" s="4">
         <v>78.400000000000006</v>
       </c>
-      <c r="I13" s="3">
+      <c r="I13" s="5">
         <v>42.8</v>
       </c>
     </row>
@@ -836,187 +845,187 @@
       <c r="A14">
         <v>2007</v>
       </c>
-      <c r="B14">
+      <c r="B14" s="6">
         <v>20</v>
       </c>
-      <c r="C14">
+      <c r="C14" s="6">
         <v>22.2</v>
       </c>
-      <c r="D14">
+      <c r="D14" s="6">
         <v>17.8</v>
       </c>
-      <c r="E14" s="7">
+      <c r="E14" s="9">
         <v>0.24343000000000001</v>
       </c>
       <c r="F14">
         <v>466.1</v>
       </c>
-      <c r="G14" s="2">
+      <c r="G14" s="4">
         <v>58.8</v>
       </c>
-      <c r="H14" s="2">
+      <c r="H14" s="4">
         <v>79.599999999999994</v>
       </c>
-      <c r="I14" s="3">
+      <c r="I14" s="5">
         <v>42</v>
       </c>
-      <c r="K14" s="2"/>
-      <c r="L14" s="2"/>
-      <c r="M14" s="2"/>
+      <c r="K14" s="1"/>
+      <c r="L14" s="1"/>
+      <c r="M14" s="1"/>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A15">
         <v>2006</v>
       </c>
-      <c r="E15" s="7">
+      <c r="B15" s="6"/>
+      <c r="C15" s="6"/>
+      <c r="D15" s="6"/>
+      <c r="E15" s="9">
         <v>0.23258999999999999</v>
       </c>
       <c r="F15">
         <v>124.1</v>
       </c>
-      <c r="G15" s="2">
+      <c r="G15" s="4">
         <v>59.2</v>
       </c>
-      <c r="H15" s="2">
+      <c r="H15" s="4">
         <v>82.6</v>
       </c>
-      <c r="I15" s="3">
+      <c r="I15" s="5">
         <v>40.6</v>
       </c>
-      <c r="K15" s="2"/>
-      <c r="L15" s="2"/>
-      <c r="M15" s="2"/>
+      <c r="K15" s="1"/>
+      <c r="L15" s="1"/>
+      <c r="M15" s="1"/>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A16">
         <v>2005</v>
       </c>
-      <c r="B16">
+      <c r="B16" s="6">
         <v>21.2</v>
       </c>
-      <c r="C16">
+      <c r="C16" s="6">
         <v>23.4</v>
       </c>
-      <c r="D16">
+      <c r="D16" s="6">
         <v>22.2</v>
       </c>
-      <c r="E16" s="7">
+      <c r="E16" s="9">
         <v>0.22914999999999999</v>
       </c>
-      <c r="G16" s="2">
+      <c r="G16" s="4">
         <v>58.4</v>
       </c>
-      <c r="H16" s="2">
+      <c r="H16" s="4">
         <v>80.900000000000006</v>
       </c>
-      <c r="I16" s="3">
+      <c r="I16" s="5">
         <v>40.299999999999997</v>
       </c>
-      <c r="J16" s="2"/>
-      <c r="K16" s="2"/>
-      <c r="M16" s="2"/>
+      <c r="J16" s="1"/>
+      <c r="K16" s="1"/>
+      <c r="M16" s="1"/>
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A17">
         <v>2004</v>
       </c>
-      <c r="B17">
+      <c r="B17" s="6">
         <v>21.3</v>
       </c>
-      <c r="C17">
+      <c r="C17" s="6">
         <v>21.7</v>
       </c>
-      <c r="D17">
+      <c r="D17" s="6">
         <v>19.8</v>
       </c>
-      <c r="E17" s="9">
+      <c r="E17" s="10">
         <v>0.22353000000000001</v>
       </c>
-      <c r="G17">
+      <c r="G17" s="6">
         <v>58.9</v>
       </c>
-      <c r="H17">
+      <c r="H17" s="6">
         <v>83.8</v>
       </c>
-      <c r="I17">
+      <c r="I17" s="6">
         <v>38.9</v>
       </c>
-      <c r="J17" s="2"/>
-      <c r="K17" s="2"/>
-      <c r="M17" s="2"/>
+      <c r="J17" s="1"/>
+      <c r="K17" s="1"/>
+      <c r="M17" s="1"/>
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A18">
         <v>2001</v>
       </c>
-      <c r="B18">
+      <c r="B18" s="6">
         <v>22.3</v>
       </c>
-      <c r="C18">
+      <c r="C18" s="6">
         <v>24.2</v>
       </c>
-      <c r="D18">
+      <c r="D18" s="6">
         <v>18</v>
       </c>
-      <c r="E18" s="7">
+      <c r="E18" s="9">
         <v>0.20644999999999999</v>
       </c>
-      <c r="G18">
+      <c r="G18" s="6">
         <v>56.8</v>
       </c>
-      <c r="H18">
+      <c r="H18" s="6">
         <v>83</v>
       </c>
-      <c r="I18">
+      <c r="I18" s="6">
         <v>36.299999999999997</v>
       </c>
-      <c r="J18" s="2"/>
-      <c r="K18" s="2"/>
-      <c r="M18" s="2"/>
+      <c r="J18" s="1"/>
+      <c r="K18" s="1"/>
+      <c r="M18" s="1"/>
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A19">
         <v>2000</v>
       </c>
-      <c r="B19">
+      <c r="B19" s="6">
         <v>24.5</v>
       </c>
-      <c r="C19">
+      <c r="C19" s="6">
         <v>26.5</v>
       </c>
-      <c r="D19">
+      <c r="D19" s="6">
         <v>22.5</v>
       </c>
-      <c r="E19" s="7">
+      <c r="E19" s="9">
         <v>0.19481000000000001</v>
       </c>
-      <c r="G19" s="2">
+      <c r="G19" s="4">
         <v>57.4</v>
       </c>
-      <c r="H19" s="2">
+      <c r="H19" s="4">
         <v>84.9</v>
       </c>
-      <c r="I19" s="3">
+      <c r="I19" s="5">
         <v>36.200000000000003</v>
       </c>
-      <c r="J19" s="2"/>
-      <c r="K19" s="2"/>
-      <c r="M19" s="2"/>
+      <c r="J19" s="1"/>
+      <c r="K19" s="1"/>
+      <c r="M19" s="1"/>
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="J20" s="2"/>
-      <c r="K20" s="2"/>
-      <c r="M20" s="2"/>
+      <c r="J20" s="1"/>
+      <c r="K20" s="1"/>
+      <c r="M20" s="1"/>
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="K21" s="2"/>
-      <c r="M21" s="2"/>
+      <c r="K21" s="1"/>
+      <c r="M21" s="1"/>
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="K22" s="2"/>
-    </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="C25" s="10"/>
+      <c r="K22" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>